<commit_message>
Update Excel schedule template columns
</commit_message>
<xml_diff>
--- a/assets/mau-lich-excel.xlsx
+++ b/assets/mau-lich-excel.xlsx
@@ -398,14 +398,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="36.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -419,12 +421,18 @@
         <v>loai</v>
       </c>
       <c r="D1" t="str">
-        <v>bat_dau</v>
+        <v>ngay_bat_dau</v>
       </c>
       <c r="E1" t="str">
-        <v>ket_thuc</v>
+        <v>gio_bat_dau</v>
       </c>
       <c r="F1" t="str">
+        <v>ngay_ket_thuc</v>
+      </c>
+      <c r="G1" t="str">
+        <v>gio_ket_thuc</v>
+      </c>
+      <c r="H1" t="str">
         <v>nhac_truoc_phut</v>
       </c>
     </row>
@@ -439,12 +447,18 @@
         <v>meeting</v>
       </c>
       <c r="D2" t="str">
-        <v>01/05/2026 09:00</v>
+        <v>01/05/2026</v>
       </c>
       <c r="E2" t="str">
-        <v>01/05/2026 10:00</v>
-      </c>
-      <c r="F2">
+        <v>09:00</v>
+      </c>
+      <c r="F2" t="str">
+        <v>01/05/2026</v>
+      </c>
+      <c r="G2" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="H2">
         <v>30</v>
       </c>
     </row>
@@ -459,12 +473,18 @@
         <v>task</v>
       </c>
       <c r="D3" t="str">
-        <v>02/05/2026 20:00</v>
+        <v>02/05/2026</v>
       </c>
       <c r="E3" t="str">
-        <v>02/05/2026 21:00</v>
-      </c>
-      <c r="F3">
+        <v>20:00</v>
+      </c>
+      <c r="F3" t="str">
+        <v>02/05/2026</v>
+      </c>
+      <c r="G3" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="H3">
         <v>60</v>
       </c>
     </row>
@@ -479,27 +499,33 @@
         <v>event</v>
       </c>
       <c r="D4" t="str">
-        <v>03/05/2026 14:00</v>
+        <v>03/05/2026</v>
       </c>
       <c r="E4" t="str">
-        <v>03/05/2026 16:00</v>
-      </c>
-      <c r="F4">
+        <v>14:00</v>
+      </c>
+      <c r="F4" t="str">
+        <v>03/05/2026</v>
+      </c>
+      <c r="G4" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="H4">
         <v>120</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <cols>
-    <col min="1" max="1" width="90.83203125" customWidth="1"/>
+    <col min="1" max="1" width="100.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -509,7 +535,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Cot bat buoc: tieu_de, loai, bat_dau, ket_thuc</v>
+        <v>Cot bat buoc: tieu_de, loai, ngay_bat_dau, gio_bat_dau, ngay_ket_thuc, gio_ket_thuc</v>
       </c>
     </row>
     <row r="3">
@@ -524,17 +550,27 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Dinh dang thoi gian khuyen dung: DD/MM/YYYY HH:mm, vi du 01/05/2026 09:00</v>
+        <v>Dinh dang ngay khuyen dung: DD/MM/YYYY hoac YYYY-MM-DD, vi du 01/05/2026</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Dinh dang gio khuyen dung: HH:mm, vi du 09:00</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>File cu dung bat_dau va ket_thuc dang DD/MM/YYYY HH:mm van duoc ho tro</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Sau khi dien xong, gui file .xlsx len Mezon va go *them-lich-excel</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>